<commit_message>
Update attractions export to 10 pages and add capture video
Co-authored-by: 吴志中 <wuzhizhong1@xdf.cn>
</commit_message>
<xml_diff>
--- a/attractionsForAgent.xlsx
+++ b/attractionsForAgent.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B151"/>
+  <dimension ref="A1:B300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1928,6 +1928,1496 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>中央大街步行街</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>印象丽江</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>崇圣寺三塔</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>文殊院</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>香港西贡</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>广州地铁</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>上海城市历史发展陈列馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>杭州宋城</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Beijing Airport Layover Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>鹿回头公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>狮子林</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>陈家祠</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>网师园</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>中国丽江古城</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>798艺术区</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>香港海事博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>东方明珠</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>崂山自然风景区</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>汉阳陵</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>峨眉山</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>同里古镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>豫园</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>大馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>云南石林地质公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>天一阁</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>西湖花港观鱼公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>金茂大厦</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>回坊风情街</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>花城广场</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>颐和园佛香阁</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>平江路</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>虎丘</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>青海湖</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>香港文化博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>太阳岛</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>鸣沙山</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>玉佛禅寺</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>凤凰古城</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>昆明龙门</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>金沙遗址博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>中华恐龙园</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>明孝陵</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>郑家大屋</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>旧城</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Happy Dragon Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>南京城墙(明城墙)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>珠海长隆海洋王国</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>新濠天地</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>周庄水乡</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Alex's Epic Xian的一日游</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>澳门历史城区</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>留园</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>香港历史博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>陕西历史博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>苏州博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>八大关</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>午门</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>珠穆朗玛峰基地营</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>两江四湖景区</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>长洲岛</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>白云山</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>峨眉山金顶</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>澳门大熊猫馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>朱家角古镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>扎什伦布寺</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>古北水镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>武汉东湖</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>大雁塔</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>锦绣中华·民俗村</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>大雁塔北广场</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>青岛啤酒博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>西塘古镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>沙面岛</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>黄龙名胜风景区</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>尖沙咀海滨长廊</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>星海广场</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>故宫九龙壁</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Guangzhou Private Local Tour Guide-Lorena</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>上海人文历史地貌区</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>复兴公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>岳麓山</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>大澳</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>外滩城市雕塑群</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>广州图书馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>大芬油画村</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>趵突泉公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>南丫岛</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>南普陀寺</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>金鸡湖</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>九龙公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Travel Beijing Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>三清山</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>SoHo 荷南美食区</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>后海</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>普陀山</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>COCO PARK</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>西安博物院</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>冈仁波齐峰</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>赤柱</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Beijing Impression Tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>厦门大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>孔庙和国子监博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>成都人民公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>束河古镇</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>China Educational Tours</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>石室圣心大教堂</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>杜甫草堂</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>圆明园</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>祖庙</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>珠江</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>上海虹桥火车站</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>元阳梯田</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>鸟巢(国家体育场)</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>北京欢乐谷</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>路环岛</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>深圳地铁</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>尖东</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>苏州古运河</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>香港科学馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>南京总统府</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>鼓浪屿</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>澳门旅游塔会展娱乐中心</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>沈阳故宫</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>中国国家博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>圣保罗大教堂遗址(大三巴牌坊)</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>平安寨</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Elysian Tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>澳门博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>西望洋主教堂</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>丽江木府</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>田子坊</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>旺角</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>西溪湿地公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>日月塔</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>洱海湖</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>九龙城寨公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>翠湖</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>洪崖洞</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>拙政园</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>黄大仙祠</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>天津之眼摩天轮</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>三亚珠江南田温泉</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>大明湖公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>三峡博物馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>世纪公园</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>前门大街商业街</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>芦笛岩</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>东望洋炮台</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>海港城</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>